<commit_message>
MDM_HQ: BP auth fix (F_KNA1_GRP/F_LFA1_GRP) as automatic rule, retest 18/18 PASS, layout synced with built state
</commit_message>
<xml_diff>
--- a/output/MDM_HQ/MDM_HQ_Layout.xlsx
+++ b/output/MDM_HQ/MDM_HQ_Layout.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="234">
   <si>
     <t>End-user layout proposition</t>
   </si>
@@ -68,7 +68,7 @@
     <t>Design status</t>
   </si>
   <si>
-    <t>PROPOSAL</t>
+    <t>BUILT_AND_TESTED</t>
   </si>
   <si>
     <t>Space</t>
@@ -104,7 +104,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-10-20T15:48:54.264Z</t>
+    <t>2026-10-21T13:31:12.955Z</t>
   </si>
   <si>
     <t>Space – technical name</t>
@@ -257,7 +257,7 @@
     <t>SAP_TC_CA_BP_BE_APPS (S4CMD)</t>
   </si>
   <si>
-    <t>→ custom catalog</t>
+    <t>Z_VOT_BEMIND_BC_MDM_HQ</t>
   </si>
   <si>
     <t>FULL (Create/Update/Delete)</t>
@@ -296,7 +296,7 @@
     <t>/UI2/PB_C_TM TCODE=MM41 PARENTID=X-SAP-UI2-ADCAT:SAP_TC_RFM_MD_ITM_BE_APPS:S4RFM</t>
   </si>
   <si>
-    <t>Change Article</t>
+    <t>Maintain Article</t>
   </si>
   <si>
     <t>MM42</t>
@@ -383,7 +383,7 @@
     <t>/UI2/PB_C_TM TCODE=ME13 PARENTID=X-SAP-UI2-ADCAT:SAP_TC_PRC_BE_APPS:S4PRC; title TSTCT</t>
   </si>
   <si>
-    <t>MDG: Export Master Data</t>
+    <t>Export Master Data - Products</t>
   </si>
   <si>
     <t>F3251</t>
@@ -404,13 +404,13 @@
     <t>Export Master Data</t>
   </si>
   <si>
-    <t>Component mdm.cmd.cmpexportfiles1 matches BSP MD_CMPEXPFILES1 of the F3251 package. Catalog CMP_MONPROCS chosen (generic CMD processes; QLTY_EVAL is data-quality specific).</t>
+    <t>Component mdm.cmd.cmpexportfiles1 matches BSP MD_CMPEXPFILES1 of the F3251 package. Catalog CMP_MONPROCS chosen (generic CMD processes; QLTY_EVAL is data-quality specific). User decision G4: Products variant only (otc=194).</t>
   </si>
   <si>
     <t>TSTC/TSTCT F3251 'MDG: Export Master Data' in package UI_MD_CMP_EXPORT_FILE (BSP MD_CMPEXPFILES1); /UI2/PB_C_TM UI5_COMPONENT_ID=mdm.cmd.cmpexportfiles1 PARENTID=X-SAP-UI2-CATALOGPAGE:SAP_TC_CMD_CMP_MONPROCS_COMMON; also listed in SAP_BR_PRODMASTER_SPECIALIST menu (AGR_HIERT 'MDG: Export Master Data')</t>
   </si>
   <si>
-    <t>Create Material BOM</t>
+    <t>Create Bill of Material</t>
   </si>
   <si>
     <t>CS01</t>
@@ -428,7 +428,7 @@
     <t>/UI2/PB_C_TM TCODE=CS01 PARENTID=X-SAP-UI2-ADCAT:SAP_TC_SCM_PP_BE_APPS:S4PP; title TSTCT</t>
   </si>
   <si>
-    <t>Change Material BOM</t>
+    <t>Change Bill of Material</t>
   </si>
   <si>
     <t>CS02</t>
@@ -461,7 +461,7 @@
     <t>TSTC F5238 package PISE_MI_PLM_BOMMULTIMAINT -&gt; UIAD 42010AEE2A311EDB8DA5F1073F43AC1E -&gt; /UI2/PB_C_TM ID ...:SAP_TC_PLM_COMMON:42010AEE2A311EDB8DA5F1073F43AC1E_TM (component pise.mi.plm.multilevelbom)</t>
   </si>
   <si>
-    <t>Display Material BOM</t>
+    <t>Display Bill of Material</t>
   </si>
   <si>
     <t>CS03</t>
@@ -479,7 +479,7 @@
     <t>/UI2/PB_C_TM TCODE=CS03 PARENTID=X-SAP-UI2-ADCAT:SAP_TC_SCM_PP_BE_APPS:S4PP; title TSTCT</t>
   </si>
   <si>
-    <t>Display Multilevel BOM</t>
+    <t>Display Multilevel BOM Explosion</t>
   </si>
   <si>
     <t>CS12</t>
@@ -512,18 +512,21 @@
     <t>TSTC F5938 package PISE_MI_PLM_BOMCOMPARISON -&gt; UIAD 42010AEE2A311EDBB8F81D5B1219F143 -&gt; /UI2/PB_C_TM ID ...:SAP_TC_PLM_COMMON:42010AEE2A311EDBB8F81D5B1219F143_TM (component pise.mi.plm.bomcomparison)</t>
   </si>
   <si>
+    <t>Manage Prices</t>
+  </si>
+  <si>
+    <t>F4111</t>
+  </si>
+  <si>
+    <t>PricesInSales-manage</t>
+  </si>
+  <si>
+    <t>SAP_TC_CEC_SD_COMMON</t>
+  </si>
+  <si>
     <t>Manage Prices - Sales</t>
   </si>
   <si>
-    <t>F4111</t>
-  </si>
-  <si>
-    <t>PricesInSales-manage</t>
-  </si>
-  <si>
-    <t>SAP_TC_CEC_SD_COMMON</t>
-  </si>
-  <si>
     <t>App ID explicitly in target mapping information.</t>
   </si>
   <si>
@@ -554,16 +557,16 @@
     <t>VK12</t>
   </si>
   <si>
-    <t>PriceCondition-setSalesPricesMaterials</t>
+    <t>PriceCondition-changeCondition</t>
   </si>
   <si>
     <t>Change condition records</t>
   </si>
   <si>
-    <t>No generic 'change condition' intent delivered for VK12. Provisional choice; see gap G2.</t>
-  </si>
-  <si>
-    <t>/UI2/PB_C_TM TCODE=VK12 PARENTID=X-SAP-UI2-ADCAT:SAP_TC_CEC_SD_BE_APPS:S4SD (only actions found: setSalesPricesMaterials, setSalesPricesServices, setSalesTaxRates)</t>
+    <t>User decision G2: generic tile without preset condition type.</t>
+  </si>
+  <si>
+    <t>Custom target mapping PriceCondition-changeCondition -&gt; VK12 (no parameters) in Z_VOT_BEMIND_BC_MDM_HQ (user decision G2)</t>
   </si>
   <si>
     <t>Display Condition</t>
@@ -663,22 +666,19 @@
     <t>ALL</t>
   </si>
   <si>
-    <t>TO_CONFIRM</t>
+    <t>RESOLVED</t>
   </si>
   <si>
     <t>Business catalogs (tile level) could not be read: tile cache /UI2/PB_C_TILE is empty in client 120. Target mappings (technical catalogs) are all found.</t>
   </si>
   <si>
-    <t>G1 - OK to build one custom business catalog Z_VOT_BEMIND_BC_MDM_HQ (in package Z_BM_ROLESAUTHORS) with 18 tiles referencing the standard target mappings above + assign the technical catalogs to the role? (Alternative: search standard SAP_*_BC_* catalogs in the FLP Content Manager via browser before building.)</t>
-  </si>
-  <si>
-    <t>AMBIGUOUS</t>
+    <t>G1 - OK to build one custom business catalog Z_VOT_BEMIND_BC_MDM_HQ (in package Z_BM_ROLESAUTHORS) with 18 tiles referencing the standard target mappings above + assign the technical catalogs to the role? (Alternative: search standard SAP_*_BC_* catalogs in the FLP Content Manager via browser before building.) -&gt; RESOLVED</t>
   </si>
   <si>
     <t>No generic 'change condition' target mapping for VK12 in the system. Delivered intents: PriceCondition-setSalesPricesMaterials / setSalesPricesServices / setSalesTaxRates (pre-filled condition types).</t>
   </si>
   <si>
-    <t>G2 - Use PriceCondition-setSalesPricesMaterials (provisional), or create a custom target mapping PriceCondition-changeCondition -&gt; VK12 without parameters in the custom catalog (my recommendation for a generic 'Change Condition' tile)?</t>
+    <t>G2 - Use PriceCondition-setSalesPricesMaterials (provisional), or create a custom target mapping PriceCondition-changeCondition -&gt; VK12 without parameters in the custom catalog (my recommendation for a generic 'Change Condition' tile)? -&gt; RESOLVED</t>
   </si>
   <si>
     <t>MM41/MM42/MM43</t>
@@ -687,13 +687,13 @@
     <t>Two standard catalogs exist: SAP_TC_RFM_MD_ITM_BE_APPS (S4RFM, retail fashion; actions create/maintain/display) and SAP_TC_CA_PR_BE_APPS (S4CMD, cross master data; actions create/change/display).</t>
   </si>
   <si>
-    <t>G3 - Keep S4RFM (matrix says 'Retail article'), or use S4CMD?</t>
+    <t>G3 - Keep S4RFM (matrix says 'Retail article'), or use S4CMD? -&gt; RESOLVED</t>
   </si>
   <si>
     <t>F3251 'MDG: Export Master Data' belongs to Central Master Data / MDG consolidation &amp; mass processing (CMD). It needs CMD/MDG configuration to be usable; may not work in S02 demo.</t>
   </si>
   <si>
-    <t>G4 - Keep F3251 in the role (matrix requirement) even if it fails in S02 tests? (Proposed: yes, failures documented in the test report.)</t>
+    <t>G4 - Keep F3251 in the role (matrix requirement) even if it fails in S02 tests? (Proposed: yes, failures documented in the test report.) -&gt; RESOLVED</t>
   </si>
   <si>
     <t>COM1 role</t>
@@ -702,7 +702,7 @@
     <t>Derived role includes all 22 COM1 plants incl. test plants 9000/9998/9999, and only purchasing orgs assigned to COM1 (9000, 9001, PO01). Cross-company purchasing orgs (e.g. HO01 with 285 info records, blank company code) are NOT included.</t>
   </si>
   <si>
-    <t>G5 - Confirm org values for Z_VOT_BEMIND_MDM_HQ_COM1 (keep all 22 plants? add any cross-company purchasing org?)</t>
+    <t>G5 - Confirm org values for Z_VOT_BEMIND_MDM_HQ_COM1 (keep all 22 plants? add any cross-company purchasing org?) -&gt; RESOLVED</t>
   </si>
   <si>
     <t>MM43, ME13, CS03, CS12, VK13</t>
@@ -711,7 +711,7 @@
     <t>Matrix marks display transactions as FULL. They remain display by nature; FULL ACTVT (01/02/03/06) is applied to the authorisation objects of the role as a whole.</t>
   </si>
   <si>
-    <t>G6 - No action needed unless you want display-only authorisation objects restricted separately.</t>
+    <t>G6 - No action needed unless you want display-only authorisation objects restricted separately. -&gt; RESOLVED</t>
   </si>
   <si>
     <t>Test user</t>
@@ -720,7 +720,13 @@
     <t>Test user Z_VOT_BM_T1 will need FLP runtime authorisations in addition to the business role (e.g. a technical FLP role).</t>
   </si>
   <si>
-    <t>G7 - Is there a project technical FLP role to assign (e.g. Z_VOT_TECHROLE?), or should I use the SAP standard SAP_UI2_USER_700 if present?</t>
+    <t>G7 - Is there a project technical FLP role to assign (e.g. Z_VOT_TECHROLE?), or should I use the SAP standard SAP_UI2_USER_700 if present? -&gt; RESOLVED</t>
+  </si>
+  <si>
+    <t>Test T01: F_KNA1_GRP/F_LFA1_GRP had ACTVT F4 only (SU24). Fixed with ACTVT 01/02/03/06 + account group *.</t>
+  </si>
+  <si>
+    <t>Now automatic rule config.authOverrides (user decision 2026-10-21)</t>
   </si>
 </sst>
 </file>
@@ -1308,7 +1314,7 @@
         <v>27</v>
       </c>
       <c r="B18" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2467,13 +2473,13 @@
         <v>18</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2490,22 +2496,22 @@
         <v>2</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I17" s="6" t="s">
         <v>78</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K17" s="6" t="s">
         <v>80</v>
@@ -2520,13 +2526,13 @@
         <v>19</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P17" s="6" t="s">
         <v>110</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2543,22 +2549,22 @@
         <v>3</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>78</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>80</v>
@@ -2573,13 +2579,13 @@
         <v>20</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2596,22 +2602,22 @@
         <v>1</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>78</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>80</v>
@@ -2626,13 +2632,13 @@
         <v>21</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="P19" s="6" t="s">
         <v>110</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2658,71 +2664,71 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -2734,7 +2740,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2746,19 +2752,19 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2766,16 +2772,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2783,10 +2789,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>216</v>
@@ -2803,7 +2809,7 @@
         <v>218</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>219</v>
@@ -2820,7 +2826,7 @@
         <v>123</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>221</v>
@@ -2837,7 +2843,7 @@
         <v>223</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>224</v>
@@ -2854,7 +2860,7 @@
         <v>226</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>227</v>
@@ -2871,13 +2877,30 @@
         <v>229</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>230</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>